<commit_message>
feat: agregar configuración del editor Puck, tablas de tendencias ocupacionales y conjunto de datos base
</commit_message>
<xml_diff>
--- a/api-backend/uploads/cargas-datos/base-tendencia-1.xlsx
+++ b/api-backend/uploads/cargas-datos/base-tendencia-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aprendiz\Documents\PROYECTOLO\OLO-proyect\api-backend\uploads\cargas-datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F7E9CF-1ACF-4815-A933-4BE1E37FA574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9B345A-B000-4978-AAF0-2691109A6F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="18900" windowHeight="10965" xr2:uid="{B387ECB8-FFDF-461D-9295-6A5C361B9F17}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="45">
   <si>
     <t>Nivel Ocupacional</t>
   </si>
@@ -523,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDB72714-76A5-4B68-8E00-474EE04C9399}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
@@ -1154,6 +1154,32 @@
         <v>36</v>
       </c>
     </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25">
+        <v>6211</v>
+      </c>
+      <c r="D25" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25">
+        <v>10</v>
+      </c>
+      <c r="F25">
+        <v>20</v>
+      </c>
+      <c r="G25">
+        <v>2020</v>
+      </c>
+      <c r="H25" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>